<commit_message>
Fix visitor_email field type: email → text with regex constraint
KoboToolbox does not render the 'email' XLSForm type; changing to 'text'
with a regex constraint makes the field appear and validates the format.

https://claude.ai/code/session_01MEjaAcBuyGtmaZejYHGrh4
</commit_message>
<xml_diff>
--- a/creamos_visitors_waiver.xlsx
+++ b/creamos_visitors_waiver.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -839,7 +839,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -857,6 +857,16 @@
           <t>Correo electrónico del visitante</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ejemplo@correo.com</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>true</t>
@@ -870,6 +880,11 @@
       <c r="J17" t="inlineStr">
         <is>
           <t>Por favor ingrese un correo electrónico válido</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>regex(., '^[a-zA-Z0-9._%+\-]+@[a-zA-Z0-9.\-]+\.[a-zA-Z]{2,}$')</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update newsletter question to be more welcoming
https://claude.ai/code/session_01MEjaAcBuyGtmaZejYHGrh4
</commit_message>
<xml_diff>
--- a/creamos_visitors_waiver.xlsx
+++ b/creamos_visitors_waiver.xlsx
@@ -901,12 +901,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Add me to your newsletter (We promise we don't spam)</t>
+          <t>Would you like to receive our newsletter? (We promise we will not spam you)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Agrégame a tu lista de correo (prometo que no te enviaremos spam)</t>
+          <t>¿Te gustaría recibir nuestro boletín informativo? (Prometemos no enviarte spam)</t>
         </is>
       </c>
     </row>

</xml_diff>